<commit_message>
chore(outputs): republish the four-question deliverables
Regenerated from the current code: Question 1 with its default reserve sensitivity,
Questions 2 to 4 from a single run whose Question 3 carries no partition
constraint, and a Question 4 that enumerates every partition without truncation
under the transport-sortie merge rule.

The superseded run01/run02/run03/review_run01 directories, whose communication
certificate predates audit_version exact_dem_interval_v2, are removed; the only
retained search record is run01, and outputs/unified/final/REPORT.md documents
the scope, the resource gaps of both partitions and the reproduction commands.
</commit_message>
<xml_diff>
--- a/outputs/unified/final/q2/problem2_submission.xlsx
+++ b/outputs/unified/final/q2/problem2_submission.xlsx
@@ -1303,7 +1303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="2"/>
   <cols>
     <col width="12" customWidth="1" style="3" min="1" max="2"/>
@@ -1361,22 +1361,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>P00001</t>
+          <t>P00026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U05</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>C-B01</t>
+          <t>B-B01</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1384,35 +1384,35 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>O01→S001→O01</t>
+          <t>O01→S015→O01</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1561.427</v>
+        <v>1829.574</v>
       </c>
       <c r="H2" t="n">
-        <v>2.926237</v>
+        <v>2.310846</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P00002</t>
+          <t>P00030</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>U08</t>
+          <t>U06</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>C-B02</t>
+          <t>B-B02</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1420,25 +1420,25 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>O01→S001→O01</t>
+          <t>O01→S008→O01</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1627.427</v>
+        <v>1905.89</v>
       </c>
       <c r="H3" t="n">
-        <v>3.004662</v>
+        <v>2.773426</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P00009</t>
+          <t>P00052</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U08</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1452,75 +1452,75 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>3976</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>O01→S004→O01</t>
+          <t>O01→S005→O01</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>6281.185</v>
+        <v>1748.046</v>
       </c>
       <c r="H4" t="n">
-        <v>6.176859</v>
+        <v>3.801897</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>P00014</t>
+          <t>P00057</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>U06</t>
+          <t>U04</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>B-B04</t>
+          <t>A-B04</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2196</v>
+        <v>0</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>O01→S009→O01</t>
+          <t>O01→S007→O01</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>3756.78</v>
+        <v>1727.319</v>
       </c>
       <c r="H5" t="n">
-        <v>2.102431</v>
+        <v>1.905043</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>P00020</t>
+          <t>P00071</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>U05</t>
+          <t>U03</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>B-B01</t>
+          <t>A-B03</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1528,169 +1528,169 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>O01→S012→O01</t>
+          <t>O01→S010→O01</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1923.801</v>
+        <v>1653.854</v>
       </c>
       <c r="H6" t="n">
-        <v>2.755193</v>
+        <v>1.9525</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>P00024</t>
+          <t>P00134</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>U05</t>
+          <t>U01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>B-B03</t>
+          <t>A-B01</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1924</v>
+        <v>0</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>O01→S014→O01</t>
+          <t>O01→S001→O01</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>3792.598</v>
+        <v>1192.472</v>
       </c>
       <c r="H7" t="n">
-        <v>2.137233</v>
+        <v>1.223053</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>P00026</t>
+          <t>P00355</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>U06</t>
+          <t>U02</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>B-B02</t>
+          <t>A-B02</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>4065</v>
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>O01→S015→O01</t>
+          <t>O01→S001→O01</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>5894.574</v>
+        <v>1252.472</v>
       </c>
       <c r="H8" t="n">
-        <v>2.310846</v>
+        <v>1.286052</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P00028</t>
+          <t>P00417</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>U05</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>B-B01</t>
+          <t>C-B01</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3793</v>
+        <v>0</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>O01→S008→O01</t>
+          <t>O01→S001→O01</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>5758.89</v>
+        <v>1561.427</v>
       </c>
       <c r="H9" t="n">
-        <v>2.98598</v>
+        <v>2.72845</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P00030</t>
+          <t>P00089</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>U06</t>
+          <t>U01</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>B-B02</t>
+          <t>A-B05</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>290</v>
+        <v>1192.472</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>O01→S008→O01</t>
+          <t>O01→S013→O01</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2195.89</v>
+        <v>2804.496</v>
       </c>
       <c r="H10" t="n">
-        <v>2.773426</v>
+        <v>1.957713</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>P00037</t>
+          <t>P00032</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>U04</t>
+          <t>U02</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1700,33 +1700,33 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>A-B04</t>
+          <t>A-B06</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1252.472</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>O01→S002→O01</t>
+          <t>O01→S001→O01</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>2007.733</v>
+        <v>2564.943</v>
       </c>
       <c r="H11" t="n">
-        <v>2.929106</v>
+        <v>1.268</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P00040</t>
+          <t>P00118</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>U08</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1736,130 +1736,130 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>C-B04</t>
+          <t>C-B03</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1628</v>
+        <v>1561.427</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>O01→S002→O01</t>
+          <t>O01→S006→S007→O01</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>3739.008</v>
+        <v>3975.206</v>
       </c>
       <c r="H12" t="n">
-        <v>6.124988</v>
+        <v>4.288062</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P00041</t>
+          <t>P00040</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>U03</t>
+          <t>U08</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>A-B05</t>
+          <t>C-B04</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3943</v>
+        <v>1748.046</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>O01→S003→O01</t>
+          <t>O01→S002→O01</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>6205.279</v>
+        <v>3859.054</v>
       </c>
       <c r="H13" t="n">
-        <v>2.981108</v>
+        <v>6.124988</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P00044</t>
+          <t>P00020</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>U08</t>
+          <t>U05</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>C-B01</t>
+          <t>B-B03</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>3740</v>
+        <v>1829.574</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>O01→S003→O01</t>
+          <t>O01→S012→O01</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>6175.811</v>
+        <v>3753.376</v>
       </c>
       <c r="H14" t="n">
-        <v>6.147682</v>
+        <v>2.755193</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>P00049</t>
+          <t>P00024</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>U02</t>
+          <t>U06</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>A-B04</t>
+          <t>B-B04</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>3364</v>
+        <v>1905.89</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>O01→S005→O01</t>
+          <t>O01→S014→O01</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>5059.759</v>
+        <v>3774.489</v>
       </c>
       <c r="H15" t="n">
-        <v>2.129487</v>
+        <v>2.137233</v>
       </c>
     </row>
     <row r="16">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>U02</t>
+          <t>U03</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1880,11 +1880,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>A-B02</t>
+          <t>A-B01</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>2045.798</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1892,7 +1892,7 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1312.616</v>
+        <v>3358.414</v>
       </c>
       <c r="H16" t="n">
         <v>1.309554</v>
@@ -1901,12 +1901,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>P00057</t>
+          <t>P00037</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>U01</t>
+          <t>U04</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1916,33 +1916,33 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>A-B05</t>
+          <t>A-B02</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1164</v>
+        <v>2123.998</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>O01→S007→O01</t>
+          <t>O01→S002→O01</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2891.319</v>
+        <v>4131.73</v>
       </c>
       <c r="H17" t="n">
-        <v>1.905043</v>
+        <v>2.929106</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>P00071</t>
+          <t>P00131</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>U04</t>
+          <t>U02</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1952,33 +1952,33 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>A-B02</t>
+          <t>A-B03</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2193</v>
+        <v>2717.909</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>O01→S010→O01</t>
+          <t>O01→S001→O01</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>3846.854</v>
+        <v>3910.381</v>
       </c>
       <c r="H18" t="n">
-        <v>1.9525</v>
+        <v>1.223053</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P00077</t>
+          <t>P00128</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>U02</t>
+          <t>U01</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1988,33 +1988,33 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>A-B02</t>
+          <t>A-B04</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>5060</v>
+        <v>2804.496</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>O01→S011→O01</t>
+          <t>O01→S001→O01</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>6283.536</v>
+        <v>3996.968</v>
       </c>
       <c r="H19" t="n">
-        <v>1.155465</v>
+        <v>1.223053</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>P00080</t>
+          <t>P00049</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>U01</t>
+          <t>U03</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2024,105 +2024,105 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>A-B01</t>
+          <t>A-B06</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>3431.254</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>O01→S011→O01</t>
+          <t>O01→S005→O01</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>1163.536</v>
+        <v>5127.014</v>
       </c>
       <c r="H20" t="n">
-        <v>1.104752</v>
+        <v>2.129487</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>P00089</t>
+          <t>P00028</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>U03</t>
+          <t>U05</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>A-B01</t>
+          <t>B-B01</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1984</v>
+        <v>3753.376</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>O01→S013→O01</t>
+          <t>O01→S008→O01</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>3596.025</v>
+        <v>5719.266</v>
       </c>
       <c r="H21" t="n">
-        <v>1.957713</v>
+        <v>2.98598</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>P00107</t>
+          <t>P00014</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>U04</t>
+          <t>U06</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>A-B06</t>
+          <t>B-B02</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>4038</v>
+        <v>3774.489</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>O01→S013→S010→O01</t>
+          <t>O01→S009→O01</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>6047.993</v>
+        <v>5335.268</v>
       </c>
       <c r="H22" t="n">
-        <v>2.246366</v>
+        <v>2.102431</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>P00118</t>
+          <t>P00044</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>U07</t>
+          <t>U08</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2132,33 +2132,33 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>C-B03</t>
+          <t>C-B01</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1562</v>
+        <v>3859.054</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>O01→S006→S007→O01</t>
+          <t>O01→S003→O01</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>3975.779</v>
+        <v>6294.865</v>
       </c>
       <c r="H23" t="n">
-        <v>4.288062</v>
+        <v>6.147682</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>P00236</t>
+          <t>P00041</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>U01</t>
+          <t>U02</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2168,69 +2168,69 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>A-B01</t>
+          <t>A-B05</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>4663</v>
+        <v>3910.381</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>O01→S005→O01</t>
+          <t>O01→S003→O01</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>6298.759</v>
+        <v>6172.659</v>
       </c>
       <c r="H24" t="n">
-        <v>2.093988</v>
+        <v>2.981108</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P00239</t>
+          <t>P00009</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>U01</t>
+          <t>U07</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>A-B03</t>
+          <t>C-B02</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>2892</v>
+        <v>3975.206</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>O01→S005→O01</t>
+          <t>O01→S004→O01</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>4527.759</v>
+        <v>6280.392</v>
       </c>
       <c r="H25" t="n">
-        <v>2.093988</v>
+        <v>6.176859</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>P00242</t>
+          <t>P00107</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>U02</t>
+          <t>U01</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2240,58 +2240,94 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>A-B06</t>
+          <t>A-B01</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1313</v>
+        <v>4236.729</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>O01→S005→O01</t>
+          <t>O01→S013→S010→O01</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>2948.759</v>
+        <v>6246.723</v>
       </c>
       <c r="H26" t="n">
-        <v>2.038021</v>
+        <v>2.246366</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>P00245</t>
+          <t>P00077</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>U04</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>A-B03</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>4763.707</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>O01→S011→O01</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>5987.243</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1.155465</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>P00080</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>U03</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>A-B03</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>O01→S005→O01</t>
-        </is>
-      </c>
-      <c r="G27" t="n">
-        <v>1635.759</v>
-      </c>
-      <c r="H27" t="n">
-        <v>2.02365</v>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>A-B04</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>5127.014</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>O01→S011→O01</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>6290.549</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1.104752</v>
       </c>
     </row>
   </sheetData>
@@ -2339,272 +2375,272 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>S001-MED-01</t>
+          <t>S015-MED-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>P00001</t>
+          <t>P00026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S015</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1248.898</v>
+        <v>1218.227</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>S001-MED-02</t>
+          <t>S015-WAT-01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>P00001</t>
+          <t>P00026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S015</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1248.898</v>
+        <v>1218.227</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>S001-WAT-01</t>
+          <t>S015-FOD-01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>P00001</t>
+          <t>P00026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S015</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1248.898</v>
+        <v>1218.227</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>S001-WAT-02</t>
+          <t>S008-WAT-02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P00001</t>
+          <t>P00030</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1248.898</v>
+        <v>1233.172</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>S001-WAT-03</t>
+          <t>S008-HYG-01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>P00001</t>
+          <t>P00030</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1248.898</v>
+        <v>1233.172</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>S001-WAT-04</t>
+          <t>S005-WAT-02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>P00001</t>
+          <t>P00052</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1248.898</v>
+        <v>1242.658</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>S001-WAT-05</t>
+          <t>S005-WAT-03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>P00001</t>
+          <t>P00052</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1248.898</v>
+        <v>1242.658</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>S001-WAT-06</t>
+          <t>S005-FOD-01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>P00002</t>
+          <t>P00052</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1314.898</v>
+        <v>1242.658</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>S001-WAT-07</t>
+          <t>S005-HYG-01</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>P00002</t>
+          <t>P00052</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1314.898</v>
+        <v>1242.658</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>S001-WAT-08</t>
+          <t>S007-MED-01</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>P00002</t>
+          <t>P00057</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1314.898</v>
+        <v>1141.299</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>S001-FOD-01</t>
+          <t>S007-WAT-01</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>P00002</t>
+          <t>P00057</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1314.898</v>
+        <v>1141.299</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>S001-FOD-02</t>
+          <t>S010-MED-01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>P00002</t>
+          <t>P00071</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S010</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1314.898</v>
+        <v>1104.463</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>S001-FOD-03</t>
+          <t>S010-WAT-01</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>P00002</t>
+          <t>P00071</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>S010</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1314.898</v>
+        <v>1104.463</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>S001-HYG-01</t>
+          <t>S001-WAT-04</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>P00002</t>
+          <t>P00134</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2613,18 +2649,18 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1314.898</v>
+        <v>849.359</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>S001-HYG-02</t>
+          <t>S001-WAT-05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>P00002</t>
+          <t>P00355</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2633,478 +2669,478 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1314.898</v>
+        <v>909.359</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>S004-MED-01</t>
+          <t>S001-FOD-01</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>P00009</t>
+          <t>P00355</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5561.563</v>
+        <v>909.359</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>S004-WAT-01</t>
+          <t>S001-WAT-06</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>P00009</t>
+          <t>P00417</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>5561.563</v>
+        <v>1248.898</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>S004-WAT-02</t>
+          <t>S001-WAT-07</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>P00009</t>
+          <t>P00417</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>5561.563</v>
+        <v>1248.898</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>S004-WAT-03</t>
+          <t>S001-WAT-08</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>P00009</t>
+          <t>P00417</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>5561.563</v>
+        <v>1248.898</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>S004-FOD-01</t>
+          <t>S001-FOD-02</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>P00009</t>
+          <t>P00417</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>5561.563</v>
+        <v>1248.898</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>S004-HYG-01</t>
+          <t>S001-FOD-03</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>P00009</t>
+          <t>P00417</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>5561.563</v>
+        <v>1248.898</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>S009-MED-01</t>
+          <t>S001-HYG-01</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>P00014</t>
+          <t>P00417</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>S009</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>3287.98</v>
+        <v>1248.898</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>S009-WAT-01</t>
+          <t>S001-HYG-02</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>P00014</t>
+          <t>P00417</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>S009</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3287.98</v>
+        <v>1248.898</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>S009-FOD-01</t>
+          <t>S013-MED-01</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>P00014</t>
+          <t>P00089</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>S009</t>
+          <t>S013</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>3287.98</v>
+        <v>2276.017</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>S012-MED-01</t>
+          <t>S013-WAT-01</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>P00020</t>
+          <t>P00089</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>S012</t>
+          <t>S013</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1271.831</v>
+        <v>2276.017</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>S012-WAT-01</t>
+          <t>S001-MED-01</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>P00020</t>
+          <t>P00032</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>S012</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1271.831</v>
+        <v>2221.831</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>S012-FOD-01</t>
+          <t>S001-MED-02</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>P00020</t>
+          <t>P00032</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>S012</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1271.831</v>
+        <v>2221.831</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>S014-MED-01</t>
+          <t>S001-WAT-01</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>P00024</t>
+          <t>P00032</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>S014</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>3165.856</v>
+        <v>2221.831</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>S014-WAT-01</t>
+          <t>S006-WAT-02</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>P00024</t>
+          <t>P00118</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>S014</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>3165.856</v>
+        <v>2728.504</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>S014-FOD-01</t>
+          <t>S006-WAT-03</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>P00024</t>
+          <t>P00118</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>S014</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>3165.856</v>
+        <v>2728.504</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>S015-MED-01</t>
+          <t>S006-FOD-01</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>P00026</t>
+          <t>P00118</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>S015</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>5283.227</v>
+        <v>2728.504</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>S015-WAT-01</t>
+          <t>S006-HYG-01</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>P00026</t>
+          <t>P00118</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>S015</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>5283.227</v>
+        <v>2728.504</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>S015-FOD-01</t>
+          <t>S007-WAT-02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>P00026</t>
+          <t>P00118</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>S015</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5283.227</v>
+        <v>3415.425</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>S008-MED-01</t>
+          <t>S007-FOD-01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>P00028</t>
+          <t>P00118</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>S008</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5086.172</v>
+        <v>3415.425</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>S008-WAT-01</t>
+          <t>S007-HYG-01</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>P00028</t>
+          <t>P00118</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>S008</t>
+          <t>S007</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>5086.172</v>
+        <v>3415.425</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>S008-FOD-01</t>
+          <t>S002-WAT-02</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>P00028</t>
+          <t>P00040</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>S008</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>5086.172</v>
+        <v>3236.96</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>S008-WAT-02</t>
+          <t>S002-WAT-03</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>P00030</t>
+          <t>P00040</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>S008</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1523.172</v>
+        <v>3236.96</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>S008-HYG-01</t>
+          <t>S002-WAT-04</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>P00030</t>
+          <t>P00040</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>S008</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1523.172</v>
+        <v>3236.96</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>S002-MED-01</t>
+          <t>S002-FOD-01</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>P00037</t>
+          <t>P00040</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3113,18 +3149,18 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1285.806</v>
+        <v>3236.96</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>S002-WAT-01</t>
+          <t>S002-FOD-02</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>P00037</t>
+          <t>P00040</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -3133,13 +3169,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1285.806</v>
+        <v>3236.96</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>S002-WAT-02</t>
+          <t>S002-HYG-01</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3153,273 +3189,273 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>3116.914</v>
+        <v>3236.96</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>S002-WAT-03</t>
+          <t>S012-MED-01</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>P00040</t>
+          <t>P00020</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S012</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3116.914</v>
+        <v>3101.405</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>S002-WAT-04</t>
+          <t>S012-WAT-01</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>P00040</t>
+          <t>P00020</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S012</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>3116.914</v>
+        <v>3101.405</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>S002-FOD-01</t>
+          <t>S012-FOD-01</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>P00040</t>
+          <t>P00020</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S012</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>3116.914</v>
+        <v>3101.405</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>S002-FOD-02</t>
+          <t>S014-MED-01</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>P00040</t>
+          <t>P00024</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S014</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>3116.914</v>
+        <v>3147.746</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>S002-HYG-01</t>
+          <t>S014-WAT-01</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>P00040</t>
+          <t>P00024</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>S014</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>3116.914</v>
+        <v>3147.746</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>S003-MED-01</t>
+          <t>S014-FOD-01</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>P00041</t>
+          <t>P00024</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S014</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>5352.113</v>
+        <v>3147.746</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>S003-WAT-01</t>
+          <t>S006-MED-01</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>P00041</t>
+          <t>P00053</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>5352.113</v>
+        <v>2980.869</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>S003-WAT-02</t>
+          <t>S006-WAT-01</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>P00044</t>
+          <t>P00053</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>5385.365</v>
+        <v>2980.869</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>S003-WAT-03</t>
+          <t>S002-MED-01</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>P00044</t>
+          <t>P00037</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>5385.365</v>
+        <v>3409.804</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>S003-WAT-04</t>
+          <t>S002-WAT-01</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>P00044</t>
+          <t>P00037</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S002</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>5385.365</v>
+        <v>3409.804</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>S003-FOD-01</t>
+          <t>S001-WAT-03</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>P00044</t>
+          <t>P00131</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>5385.365</v>
+        <v>3567.268</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>S003-FOD-02</t>
+          <t>S001-WAT-02</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>P00044</t>
+          <t>P00128</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S001</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>5385.365</v>
+        <v>3653.855</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>S003-HYG-01</t>
+          <t>S005-MED-01</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>P00044</t>
+          <t>P00049</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>5385.365</v>
+        <v>4561.891</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>S005-MED-01</t>
+          <t>S005-WAT-01</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3433,507 +3469,507 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>4494.636</v>
+        <v>4561.891</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>S005-WAT-01</t>
+          <t>S008-MED-01</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>P00049</t>
+          <t>P00028</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>S005</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>4494.636</v>
+        <v>5046.547</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>S006-MED-01</t>
+          <t>S008-WAT-01</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>P00053</t>
+          <t>P00028</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>935.071</v>
+        <v>5046.547</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>S006-WAT-01</t>
+          <t>S008-FOD-01</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>P00053</t>
+          <t>P00028</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>S008</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>935.071</v>
+        <v>5046.547</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>S007-MED-01</t>
+          <t>S009-MED-01</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>P00057</t>
+          <t>P00014</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>S007</t>
+          <t>S009</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>2305.299</v>
+        <v>4866.468</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>S007-WAT-01</t>
+          <t>S009-WAT-01</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>P00057</t>
+          <t>P00014</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>S007</t>
+          <t>S009</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>2305.299</v>
+        <v>4866.468</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>S010-MED-01</t>
+          <t>S009-FOD-01</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>P00071</t>
+          <t>P00014</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>S010</t>
+          <t>S009</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>3297.463</v>
+        <v>4866.468</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>S010-WAT-01</t>
+          <t>S003-WAT-02</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>P00071</t>
+          <t>P00044</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>S010</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>3297.463</v>
+        <v>5504.419</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S011-MED-01</t>
+          <t>S003-WAT-03</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>P00077</t>
+          <t>P00044</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>S011</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5953.955</v>
+        <v>5504.419</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>S011-WAT-01</t>
+          <t>S003-WAT-04</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>P00077</t>
+          <t>P00044</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>S011</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>5953.955</v>
+        <v>5504.419</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>S011-FOD-01</t>
+          <t>S003-FOD-01</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>P00080</t>
+          <t>P00044</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>S011</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>833.955</v>
+        <v>5504.419</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>S013-MED-01</t>
+          <t>S003-FOD-02</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>P00089</t>
+          <t>P00044</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>S013</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>3067.546</v>
+        <v>5504.419</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>S013-WAT-01</t>
+          <t>S003-HYG-01</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>P00089</t>
+          <t>P00044</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>S013</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>3067.546</v>
+        <v>5504.419</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>S010-FOD-01</t>
+          <t>S003-MED-01</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>P00107</t>
+          <t>P00041</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>S010</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>5498.603</v>
+        <v>5319.493</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>S013-FOD-01</t>
+          <t>S003-WAT-01</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>P00107</t>
+          <t>P00041</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>S013</t>
+          <t>S003</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>5091.546</v>
+        <v>5319.493</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>S006-WAT-02</t>
+          <t>S004-MED-01</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>P00118</t>
+          <t>P00009</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>2729.077</v>
+        <v>5560.769</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>S006-WAT-03</t>
+          <t>S004-WAT-01</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>P00118</t>
+          <t>P00009</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>2729.077</v>
+        <v>5560.769</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>S006-FOD-01</t>
+          <t>S004-WAT-02</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>P00118</t>
+          <t>P00009</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>2729.077</v>
+        <v>5560.769</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>S006-HYG-01</t>
+          <t>S004-WAT-03</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>P00118</t>
+          <t>P00009</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>2729.077</v>
+        <v>5560.769</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>S007-WAT-02</t>
+          <t>S004-FOD-01</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>P00118</t>
+          <t>P00009</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>S007</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>3415.998</v>
+        <v>5560.769</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>S007-FOD-01</t>
+          <t>S004-HYG-01</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>P00118</t>
+          <t>P00009</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>S007</t>
+          <t>S004</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>3415.998</v>
+        <v>5560.769</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>S007-HYG-01</t>
+          <t>S010-FOD-01</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>P00118</t>
+          <t>P00107</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>S007</t>
+          <t>S010</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>3415.998</v>
+        <v>5697.333</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>S005-WAT-02</t>
+          <t>S013-FOD-01</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>P00236</t>
+          <t>P00107</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>S005</t>
+          <t>S013</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>5733.636</v>
+        <v>5290.275</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>S005-WAT-03</t>
+          <t>S011-MED-01</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>P00239</t>
+          <t>P00077</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>S005</t>
+          <t>S011</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>3962.636</v>
+        <v>5657.662</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>S005-FOD-01</t>
+          <t>S011-WAT-01</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>P00242</t>
+          <t>P00077</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>S005</t>
+          <t>S011</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>2383.636</v>
+        <v>5657.662</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>S005-HYG-01</t>
+          <t>S011-FOD-01</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>P00245</t>
+          <t>P00080</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>S005</t>
+          <t>S011</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>1070.636</v>
+        <v>5960.968</v>
       </c>
     </row>
   </sheetData>

</xml_diff>